<commit_message>
Add CWE-1233 vulnerabilities to CWE-1245 examples vulnerability mapping
</commit_message>
<xml_diff>
--- a/CWE_Examples/CWE-1245/CWE-1245-vulnerability-mapping.xlsx
+++ b/CWE_Examples/CWE-1245/CWE-1245-vulnerability-mapping.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\parks\OneDrive\Documents\UC\Summer Research\CWE_Examples\CWE-1245\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\parks\OneDrive\Documents\UC\Summer Research\DetectRTL\CWE_Examples\CWE-1245\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2EFC5F8-ACB8-4040-B904-B505A98B1BF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCE78F3C-2C9D-4CF9-A11B-116D78C73619}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19110" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="47">
   <si>
     <t>File Name</t>
   </si>
@@ -94,14 +94,94 @@
   </si>
   <si>
     <t>Vulnerable: Deadlock in '`HOLD' state</t>
+  </si>
+  <si>
+    <t>CWE_1245_example_1_fixed_parsed.v</t>
+  </si>
+  <si>
+    <t>CWE_1245_example_2_fixed_parsed.v</t>
+  </si>
+  <si>
+    <t>CWE_1245_example_3_fixed_parsed.v</t>
+  </si>
+  <si>
+    <t>CWE_1245_example_4_fixed_parsed.v</t>
+  </si>
+  <si>
+    <t>CWE_1245_example_5_fixed_parsed.v</t>
+  </si>
+  <si>
+    <t>CWE_1245_example_6_fixed_parsed.v</t>
+  </si>
+  <si>
+    <t>CWE_1245_example_7_fixed_parsed.v</t>
+  </si>
+  <si>
+    <t>CWE_1245_example_8_fixed_parsed.v</t>
+  </si>
+  <si>
+    <t>CWE_1245_example_10_fixed_parsed.v</t>
+  </si>
+  <si>
+    <t>Detected Security Sensitive Registers</t>
+  </si>
+  <si>
+    <t>Lock Enforcment Completeness</t>
+  </si>
+  <si>
+    <t>Security Sensitive Coverage Completeness</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>Secure: No Security Sensitive Registers</t>
+  </si>
+  <si>
+    <t>fuse_req_o, fuse_addr_o, rdata</t>
+  </si>
+  <si>
+    <t>Secure: Register locks restrict unauthorized writes</t>
+  </si>
+  <si>
+    <t>Secure: All security sensitive registers covered</t>
+  </si>
+  <si>
+    <t>start, p_c, key0, state, key1, key2, key_sel, rdata</t>
+  </si>
+  <si>
+    <t>CWE_1245_example_10_vulnerable_parsed.sv</t>
+  </si>
+  <si>
+    <t>Lock Enforcement Completeness</t>
+  </si>
+  <si>
+    <t>CWE-1233 Vulnerabilities on CWE-1245 Fixed Examples</t>
+  </si>
+  <si>
+    <t>CWE-1233 Vulnerabilities on CWE-1245 Vulnerable Examples</t>
+  </si>
+  <si>
+    <t>CWE-1245 Vulnerabilities on CWE-1245 Secure Examples</t>
+  </si>
+  <si>
+    <t>CWE-1245 Vulnerabilities on CWE-1245 Vulnerable Examples</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -129,16 +209,101 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="26">
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -149,6 +314,60 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5F94C13D-904B-4ABD-9F7E-53C3DC390700}" name="Table1" displayName="Table1" ref="A2:E13" totalsRowShown="0" headerRowDxfId="19" dataDxfId="20">
+  <autoFilter ref="A2:E13" xr:uid="{5F94C13D-904B-4ABD-9F7E-53C3DC390700}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{B9661404-79CE-40A3-9E22-450B66FCA9A1}" name="File Name" dataDxfId="25"/>
+    <tableColumn id="2" xr3:uid="{C8557D32-6F96-41D5-811F-33B42706893F}" name="Case Number" dataDxfId="24"/>
+    <tableColumn id="3" xr3:uid="{EF0A8365-2E22-43CB-9B9A-1439EC7CA8E5}" name="State Coverage" dataDxfId="23"/>
+    <tableColumn id="4" xr3:uid="{0B41959F-D795-4C04-84EF-054AD8E21F8B}" name="Unreachable States" dataDxfId="22"/>
+    <tableColumn id="5" xr3:uid="{9A2B96AD-6AE4-4701-87A4-A968E160A7E1}" name="Deadlocks" dataDxfId="21"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{7E831A8D-7049-44E1-B3F8-69447E945B54}" name="Table13" displayName="Table13" ref="A16:E27" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
+  <autoFilter ref="A16:E27" xr:uid="{7E831A8D-7049-44E1-B3F8-69447E945B54}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{9D6653A0-D914-486B-AA04-6BC34EA1755E}" name="File Name" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{835B414E-60F3-4563-AE19-85BB73F98EC7}" name="Case Number" dataDxfId="15"/>
+    <tableColumn id="3" xr3:uid="{4A9AED78-B318-45AE-9A61-6224AD9CFCC4}" name="State Coverage" dataDxfId="14"/>
+    <tableColumn id="4" xr3:uid="{2B03A665-DA4A-4154-82A1-BAF7C4C383F3}" name="Unreachable States" dataDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{58544891-3CF4-4016-8E58-34CB9D6A312A}" name="Deadlocks" dataDxfId="12"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{8FF6985B-A3A9-42AA-AEF6-B56A291D5CEF}" name="Table14" displayName="Table14" ref="A30:D39" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
+  <autoFilter ref="A30:D39" xr:uid="{8FF6985B-A3A9-42AA-AEF6-B56A291D5CEF}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{A17E7B7C-3232-4045-BE8F-2D9E6A726AF1}" name="File Name" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{188FAD86-9447-4272-A61D-871D8663F137}" name="Detected Security Sensitive Registers" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{0B2F33E6-C8DD-43FA-8D0E-F822A3A4C169}" name="Lock Enforcment Completeness" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{5ED07D4F-3B09-472D-B0C7-E3A0F3C3DEFB}" name="Security Sensitive Coverage Completeness" dataDxfId="6"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{2A9C392D-FF89-44AD-98DE-902946B1E240}" name="Table2" displayName="Table2" ref="A42:D51" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
+  <autoFilter ref="A42:D51" xr:uid="{2A9C392D-FF89-44AD-98DE-902946B1E240}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{0E1CF1B3-3252-464A-AE20-BF70F2A88F80}" name="File Name" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{76F89AE4-DA27-4862-BD0F-0552818C4237}" name="Detected Security Sensitive Registers" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{3BADF4E4-8711-4EE7-8EE4-4FA5B55C4D4F}" name="Lock Enforcement Completeness" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{8F3C1F3C-844D-44E8-B298-BB925F64E915}" name="Security Sensitive Coverage Completeness" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -414,47 +633,39 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="43.77734375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="8.88671875" style="1"/>
+    <col min="2" max="2" width="14.44140625" style="1" customWidth="1"/>
     <col min="3" max="5" width="32.88671875" style="1" customWidth="1"/>
     <col min="6" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="1">
-        <v>1</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
@@ -627,7 +838,547 @@
         <v>20</v>
       </c>
     </row>
+    <row r="13" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B13" s="1">
+        <v>1</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A17" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B17" s="1">
+        <v>1</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A18" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B18" s="1">
+        <v>1</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A19" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B19" s="1">
+        <v>1</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A20" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20" s="1">
+        <v>1</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A21" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B21" s="1">
+        <v>1</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A22" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B22" s="1">
+        <v>1</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A23" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B23" s="1">
+        <v>1</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A24" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B24" s="1">
+        <v>2</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A25" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B25" s="1">
+        <v>1</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A26" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B26" s="1">
+        <v>2</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A27" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B27" s="1">
+        <v>1</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A29" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B29" s="2"/>
+      <c r="C29" s="2"/>
+      <c r="D29" s="2"/>
+    </row>
+    <row r="30" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A30" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" ht="72.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" ht="72.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A41" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B41" s="2"/>
+      <c r="C41" s="2"/>
+      <c r="D41" s="2"/>
+    </row>
+    <row r="42" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A42" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" ht="61.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D49" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" ht="61.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D50" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D51" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A15:E15"/>
+    <mergeCell ref="A41:D41"/>
+    <mergeCell ref="A29:D29"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <tableParts count="4">
+    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId4"/>
+    <tablePart r:id="rId5"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update CWE 1233 vulnerable example 2 & 8 to allow unauthorized writes Update vulnerability mappings
</commit_message>
<xml_diff>
--- a/CWE_Examples/CWE-1245/CWE-1245-vulnerability-mapping.xlsx
+++ b/CWE_Examples/CWE-1245/CWE-1245-vulnerability-mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\parks\OneDrive\Documents\UC\Summer Research\DetectRTL\CWE_Examples\CWE-1245\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCE78F3C-2C9D-4CF9-A11B-116D78C73619}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9E9F00C-DBD3-47EE-8624-E214F6C758F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19110" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -123,9 +123,6 @@
     <t>CWE_1245_example_10_fixed_parsed.v</t>
   </si>
   <si>
-    <t>Detected Security Sensitive Registers</t>
-  </si>
-  <si>
     <t>Lock Enforcment Completeness</t>
   </si>
   <si>
@@ -156,16 +153,19 @@
     <t>Lock Enforcement Completeness</t>
   </si>
   <si>
-    <t>CWE-1233 Vulnerabilities on CWE-1245 Fixed Examples</t>
-  </si>
-  <si>
-    <t>CWE-1233 Vulnerabilities on CWE-1245 Vulnerable Examples</t>
-  </si>
-  <si>
-    <t>CWE-1245 Vulnerabilities on CWE-1245 Secure Examples</t>
-  </si>
-  <si>
-    <t>CWE-1245 Vulnerabilities on CWE-1245 Vulnerable Examples</t>
+    <t>CWE-1245 Vulnerabilities in CWE-1245 Vulnerable Examples</t>
+  </si>
+  <si>
+    <t>CWE-1245 Vulnerabilities in CWE-1245 Secure Examples</t>
+  </si>
+  <si>
+    <t>CWE-1233 Vulnerabilities in CWE-1245 Vulnerable Examples</t>
+  </si>
+  <si>
+    <t>Security Sensitive Registers</t>
+  </si>
+  <si>
+    <t>CWE-1233 Vulnerabilities in CWE-1245 Fixed Examples</t>
   </si>
 </sst>
 </file>
@@ -349,7 +349,7 @@
   <autoFilter ref="A30:D39" xr:uid="{8FF6985B-A3A9-42AA-AEF6-B56A291D5CEF}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{A17E7B7C-3232-4045-BE8F-2D9E6A726AF1}" name="File Name" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{188FAD86-9447-4272-A61D-871D8663F137}" name="Detected Security Sensitive Registers" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{188FAD86-9447-4272-A61D-871D8663F137}" name="Security Sensitive Registers" dataDxfId="8"/>
     <tableColumn id="3" xr3:uid="{0B2F33E6-C8DD-43FA-8D0E-F822A3A4C169}" name="Lock Enforcment Completeness" dataDxfId="7"/>
     <tableColumn id="4" xr3:uid="{5ED07D4F-3B09-472D-B0C7-E3A0F3C3DEFB}" name="Security Sensitive Coverage Completeness" dataDxfId="6"/>
   </tableColumns>
@@ -362,7 +362,7 @@
   <autoFilter ref="A42:D51" xr:uid="{2A9C392D-FF89-44AD-98DE-902946B1E240}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{0E1CF1B3-3252-464A-AE20-BF70F2A88F80}" name="File Name" dataDxfId="3"/>
-    <tableColumn id="2" xr3:uid="{76F89AE4-DA27-4862-BD0F-0552818C4237}" name="Detected Security Sensitive Registers" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{76F89AE4-DA27-4862-BD0F-0552818C4237}" name="Security Sensitive Registers" dataDxfId="2"/>
     <tableColumn id="3" xr3:uid="{3BADF4E4-8711-4EE7-8EE4-4FA5B55C4D4F}" name="Lock Enforcement Completeness" dataDxfId="1"/>
     <tableColumn id="4" xr3:uid="{8F3C1F3C-844D-44E8-B298-BB925F64E915}" name="Security Sensitive Coverage Completeness" dataDxfId="0"/>
   </tableColumns>
@@ -644,7 +644,7 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -857,7 +857,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -1076,18 +1076,18 @@
       <c r="C29" s="2"/>
       <c r="D29" s="2"/>
     </row>
-    <row r="30" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B30" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C30" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C30" s="1" t="s">
+      <c r="D30" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
@@ -1095,13 +1095,13 @@
         <v>6</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
@@ -1109,13 +1109,13 @@
         <v>7</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
@@ -1123,13 +1123,13 @@
         <v>8</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
@@ -1137,13 +1137,13 @@
         <v>9</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
@@ -1151,13 +1151,13 @@
         <v>10</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
@@ -1165,13 +1165,13 @@
         <v>11</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="72.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
@@ -1179,13 +1179,13 @@
         <v>12</v>
       </c>
       <c r="B37" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C37" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C37" s="1" t="s">
+      <c r="D37" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="D37" s="1" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="72.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
@@ -1193,50 +1193,50 @@
         <v>13</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C38" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D38" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="D38" s="1" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" s="3" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
       <c r="D41" s="2"/>
     </row>
-    <row r="42" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1244,13 +1244,13 @@
         <v>23</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1258,13 +1258,13 @@
         <v>24</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="45" spans="1:4" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1272,13 +1272,13 @@
         <v>25</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1286,13 +1286,13 @@
         <v>26</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1300,13 +1300,13 @@
         <v>27</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="48" spans="1:4" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1314,13 +1314,13 @@
         <v>28</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="49" spans="1:4" ht="61.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -1328,13 +1328,13 @@
         <v>29</v>
       </c>
       <c r="B49" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C49" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C49" s="1" t="s">
+      <c r="D49" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="D49" s="1" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="50" spans="1:4" ht="61.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -1342,13 +1342,13 @@
         <v>30</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C50" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D50" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="D50" s="1" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="51" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -1356,13 +1356,13 @@
         <v>31</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Small modifications to vulnerability mappings
</commit_message>
<xml_diff>
--- a/CWE_Examples/CWE-1245/CWE-1245-vulnerability-mapping.xlsx
+++ b/CWE_Examples/CWE-1245/CWE-1245-vulnerability-mapping.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\parks\OneDrive\Documents\UC\Summer Research\DetectRTL\CWE_Examples\CWE-1245\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\parks\OneDrive\Documents\UC\Research\DetectRTL\CWE_Examples\CWE-1245\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9E9F00C-DBD3-47EE-8624-E214F6C758F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82692D53-9396-4D25-8EFD-2F771FDF8E87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19110" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-9690" yWindow="-16455" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="34">
   <si>
     <t>File Name</t>
   </si>
@@ -96,76 +96,37 @@
     <t>Vulnerable: Deadlock in '`HOLD' state</t>
   </si>
   <si>
-    <t>CWE_1245_example_1_fixed_parsed.v</t>
-  </si>
-  <si>
-    <t>CWE_1245_example_2_fixed_parsed.v</t>
-  </si>
-  <si>
-    <t>CWE_1245_example_3_fixed_parsed.v</t>
-  </si>
-  <si>
-    <t>CWE_1245_example_4_fixed_parsed.v</t>
-  </si>
-  <si>
-    <t>CWE_1245_example_5_fixed_parsed.v</t>
-  </si>
-  <si>
-    <t>CWE_1245_example_6_fixed_parsed.v</t>
-  </si>
-  <si>
-    <t>CWE_1245_example_7_fixed_parsed.v</t>
-  </si>
-  <si>
-    <t>CWE_1245_example_8_fixed_parsed.v</t>
-  </si>
-  <si>
-    <t>CWE_1245_example_10_fixed_parsed.v</t>
-  </si>
-  <si>
-    <t>Lock Enforcment Completeness</t>
-  </si>
-  <si>
-    <t>Security Sensitive Coverage Completeness</t>
-  </si>
-  <si>
-    <t>None</t>
-  </si>
-  <si>
-    <t>Secure: No Security Sensitive Registers</t>
-  </si>
-  <si>
-    <t>fuse_req_o, fuse_addr_o, rdata</t>
-  </si>
-  <si>
-    <t>Secure: Register locks restrict unauthorized writes</t>
-  </si>
-  <si>
-    <t>Secure: All security sensitive registers covered</t>
-  </si>
-  <si>
-    <t>start, p_c, key0, state, key1, key2, key_sel, rdata</t>
-  </si>
-  <si>
-    <t>CWE_1245_example_10_vulnerable_parsed.sv</t>
-  </si>
-  <si>
-    <t>Lock Enforcement Completeness</t>
-  </si>
-  <si>
     <t>CWE-1245 Vulnerabilities in CWE-1245 Vulnerable Examples</t>
   </si>
   <si>
     <t>CWE-1245 Vulnerabilities in CWE-1245 Secure Examples</t>
   </si>
   <si>
-    <t>CWE-1233 Vulnerabilities in CWE-1245 Vulnerable Examples</t>
-  </si>
-  <si>
-    <t>Security Sensitive Registers</t>
-  </si>
-  <si>
-    <t>CWE-1233 Vulnerabilities in CWE-1245 Fixed Examples</t>
+    <t>CWE_1245_example_1_secure_parsed.v</t>
+  </si>
+  <si>
+    <t>CWE_1245_example_2_secure_parsed.v</t>
+  </si>
+  <si>
+    <t>CWE_1245_example_3_secure_parsed.v</t>
+  </si>
+  <si>
+    <t>CWE_1245_example_4_secure_parsed.v</t>
+  </si>
+  <si>
+    <t>CWE_1245_example_5_secure_parsed.v</t>
+  </si>
+  <si>
+    <t>CWE_1245_example_6_secure_parsed.v</t>
+  </si>
+  <si>
+    <t>CWE_1245_example_7_secure_parsed.v</t>
+  </si>
+  <si>
+    <t>CWE_1245_example_8_secure_parsed.v</t>
+  </si>
+  <si>
+    <t>CWE_1245_example_10_secure_parsed.v</t>
   </si>
 </sst>
 </file>
@@ -209,58 +170,28 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="26">
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
+  <dxfs count="14">
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -317,54 +248,28 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5F94C13D-904B-4ABD-9F7E-53C3DC390700}" name="Table1" displayName="Table1" ref="A2:E13" totalsRowShown="0" headerRowDxfId="19" dataDxfId="20">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5F94C13D-904B-4ABD-9F7E-53C3DC390700}" name="Table1" displayName="Table1" ref="A2:E13" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
   <autoFilter ref="A2:E13" xr:uid="{5F94C13D-904B-4ABD-9F7E-53C3DC390700}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{B9661404-79CE-40A3-9E22-450B66FCA9A1}" name="File Name" dataDxfId="25"/>
-    <tableColumn id="2" xr3:uid="{C8557D32-6F96-41D5-811F-33B42706893F}" name="Case Number" dataDxfId="24"/>
-    <tableColumn id="3" xr3:uid="{EF0A8365-2E22-43CB-9B9A-1439EC7CA8E5}" name="State Coverage" dataDxfId="23"/>
-    <tableColumn id="4" xr3:uid="{0B41959F-D795-4C04-84EF-054AD8E21F8B}" name="Unreachable States" dataDxfId="22"/>
-    <tableColumn id="5" xr3:uid="{9A2B96AD-6AE4-4701-87A4-A968E160A7E1}" name="Deadlocks" dataDxfId="21"/>
+    <tableColumn id="1" xr3:uid="{B9661404-79CE-40A3-9E22-450B66FCA9A1}" name="File Name" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{C8557D32-6F96-41D5-811F-33B42706893F}" name="Case Number" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{EF0A8365-2E22-43CB-9B9A-1439EC7CA8E5}" name="State Coverage" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{0B41959F-D795-4C04-84EF-054AD8E21F8B}" name="Unreachable States" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{9A2B96AD-6AE4-4701-87A4-A968E160A7E1}" name="Deadlocks" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{7E831A8D-7049-44E1-B3F8-69447E945B54}" name="Table13" displayName="Table13" ref="A16:E27" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{7E831A8D-7049-44E1-B3F8-69447E945B54}" name="Table13" displayName="Table13" ref="A16:E27" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
   <autoFilter ref="A16:E27" xr:uid="{7E831A8D-7049-44E1-B3F8-69447E945B54}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{9D6653A0-D914-486B-AA04-6BC34EA1755E}" name="File Name" dataDxfId="16"/>
-    <tableColumn id="2" xr3:uid="{835B414E-60F3-4563-AE19-85BB73F98EC7}" name="Case Number" dataDxfId="15"/>
-    <tableColumn id="3" xr3:uid="{4A9AED78-B318-45AE-9A61-6224AD9CFCC4}" name="State Coverage" dataDxfId="14"/>
-    <tableColumn id="4" xr3:uid="{2B03A665-DA4A-4154-82A1-BAF7C4C383F3}" name="Unreachable States" dataDxfId="13"/>
-    <tableColumn id="5" xr3:uid="{58544891-3CF4-4016-8E58-34CB9D6A312A}" name="Deadlocks" dataDxfId="12"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{8FF6985B-A3A9-42AA-AEF6-B56A291D5CEF}" name="Table14" displayName="Table14" ref="A30:D39" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
-  <autoFilter ref="A30:D39" xr:uid="{8FF6985B-A3A9-42AA-AEF6-B56A291D5CEF}"/>
-  <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{A17E7B7C-3232-4045-BE8F-2D9E6A726AF1}" name="File Name" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{188FAD86-9447-4272-A61D-871D8663F137}" name="Security Sensitive Registers" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{0B2F33E6-C8DD-43FA-8D0E-F822A3A4C169}" name="Lock Enforcment Completeness" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{5ED07D4F-3B09-472D-B0C7-E3A0F3C3DEFB}" name="Security Sensitive Coverage Completeness" dataDxfId="6"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{2A9C392D-FF89-44AD-98DE-902946B1E240}" name="Table2" displayName="Table2" ref="A42:D51" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
-  <autoFilter ref="A42:D51" xr:uid="{2A9C392D-FF89-44AD-98DE-902946B1E240}"/>
-  <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{0E1CF1B3-3252-464A-AE20-BF70F2A88F80}" name="File Name" dataDxfId="3"/>
-    <tableColumn id="2" xr3:uid="{76F89AE4-DA27-4862-BD0F-0552818C4237}" name="Security Sensitive Registers" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{3BADF4E4-8711-4EE7-8EE4-4FA5B55C4D4F}" name="Lock Enforcement Completeness" dataDxfId="1"/>
-    <tableColumn id="4" xr3:uid="{8F3C1F3C-844D-44E8-B298-BB925F64E915}" name="Security Sensitive Coverage Completeness" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{9D6653A0-D914-486B-AA04-6BC34EA1755E}" name="File Name" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{835B414E-60F3-4563-AE19-85BB73F98EC7}" name="Case Number" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{4A9AED78-B318-45AE-9A61-6224AD9CFCC4}" name="State Coverage" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{2B03A665-DA4A-4154-82A1-BAF7C4C383F3}" name="Unreachable States" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{58544891-3CF4-4016-8E58-34CB9D6A312A}" name="Deadlocks" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -643,13 +548,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
+      <c r="A1" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -856,13 +761,13 @@
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
+      <c r="A15" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B15" s="5"/>
+      <c r="C15" s="5"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
@@ -883,13 +788,13 @@
     </row>
     <row r="17" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B17" s="1">
         <v>1</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>17</v>
@@ -900,30 +805,30 @@
     </row>
     <row r="18" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B18" s="1">
         <v>1</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>17</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B19" s="1">
         <v>1</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>17</v>
@@ -934,7 +839,7 @@
     </row>
     <row r="20" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B20" s="1">
         <v>1</v>
@@ -946,12 +851,12 @@
         <v>17</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B21" s="1">
         <v>1</v>
@@ -960,7 +865,7 @@
         <v>14</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>20</v>
@@ -968,7 +873,7 @@
     </row>
     <row r="22" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B22" s="1">
         <v>1</v>
@@ -980,12 +885,12 @@
         <v>17</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B23" s="1">
         <v>1</v>
@@ -1000,15 +905,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="24" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B24" s="1">
         <v>2</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>17</v>
@@ -1019,7 +924,7 @@
     </row>
     <row r="25" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B25" s="1">
         <v>1</v>
@@ -1034,15 +939,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="26" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B26" s="1">
         <v>2</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D26" s="1" t="s">
         <v>17</v>
@@ -1053,7 +958,7 @@
     </row>
     <row r="27" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B27" s="1">
         <v>1</v>
@@ -1065,320 +970,50 @@
         <v>17</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A29" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="B29" s="2"/>
-      <c r="C29" s="2"/>
-      <c r="D29" s="2"/>
-    </row>
-    <row r="30" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A30" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B31" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="D35" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="D36" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" ht="72.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="D37" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" ht="72.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B38" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="C38" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="D38" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B39" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C39" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="D39" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="2"/>
+      <c r="B29" s="3"/>
+      <c r="C29" s="3"/>
+      <c r="D29" s="3"/>
+    </row>
+    <row r="31" spans="1:5" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="32" spans="1:5" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="33" spans="1:4" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="34" spans="1:4" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="35" spans="1:4" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="36" spans="1:4" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="37" spans="1:4" ht="72.599999999999994" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="38" spans="1:4" ht="72.599999999999994" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="39" spans="1:4" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="40" spans="1:4" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A41" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="B41" s="2"/>
-      <c r="C41" s="2"/>
-      <c r="D41" s="2"/>
-    </row>
-    <row r="42" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A42" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B42" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C42" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="D42" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B43" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C43" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="D43" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B44" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C44" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="D44" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B45" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C45" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="D45" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B46" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C46" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="D46" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B47" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C47" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="D47" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B48" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C48" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="D48" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" ht="61.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B49" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C49" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="D49" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" ht="61.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B50" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="C50" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="D50" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="B51" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C51" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="D51" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
+    <row r="41" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="2"/>
+      <c r="B41" s="3"/>
+      <c r="C41" s="3"/>
+      <c r="D41" s="3"/>
+    </row>
+    <row r="43" spans="1:4" ht="42.6" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="44" spans="1:4" ht="42.6" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="45" spans="1:4" ht="42.6" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="46" spans="1:4" ht="42.6" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="47" spans="1:4" ht="42.6" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="48" spans="1:4" ht="42.6" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="49" ht="61.2" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="50" ht="61.2" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="51" ht="36" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="2">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A15:E15"/>
-    <mergeCell ref="A41:D41"/>
-    <mergeCell ref="A29:D29"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
-  <tableParts count="4">
+  <tableParts count="2">
     <tablePart r:id="rId2"/>
     <tablePart r:id="rId3"/>
-    <tablePart r:id="rId4"/>
-    <tablePart r:id="rId5"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>